<commit_message>
Fix default column widths
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/NullableTests.NullDisplay.verified.xlsx
+++ b/src/Excelsior.Tests/NullableTests.NullDisplay.verified.xlsx
@@ -71,8 +71,8 @@
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="23" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
     <col min="6" max="6" width="13" customWidth="1"/>
   </cols>

</xml_diff>